<commit_message>
data: 2026-06 월별 취합 (로컬 수동)
</commit_message>
<xml_diff>
--- a/data/monthly/2026-06_월별취합.xlsx
+++ b/data/monthly/2026-06_월별취합.xlsx
@@ -421,9 +421,9 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="59" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
@@ -476,7 +476,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)+파인키위효소 1개월+저당견과류바</t>
+          <t>[그레인온] 골드 카무트 브랜드밀효소G 3개월분+10포증정(총100포)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -486,7 +486,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>43,900원</t>
+          <t>24,900원</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -502,22 +502,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>멀티비타민/종합비타민</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 7입 (공식수입)</t>
+          <t>[카카오 단독 특가]센트룸 원데이팩 맨/우먼 2030 30일팩 2종 택1</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>오쏘몰</t>
+          <t>센트룸</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>34,000원</t>
+          <t>50,000원</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -538,24 +538,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>옵티젠 이뮨 멀티비타민&amp;미네랄 10입 / 1박스 (+GIFT 쇼핑백)</t>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 7입 (공식수입)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>옵티젠</t>
+          <t>오쏘몰</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>26,900원</t>
+          <t>34,000원</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -564,26 +564,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[한끼통살] 닭가슴살 한달 식단패키지 30팩+(증정)보냉백</t>
+          <t>물에 타먹는 발포형 무설탕 이온음료 요헤미티 워터 네가지 맛 4통(40정)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>요헤미티</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>45,900원</t>
+          <t>34,000원</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -600,7 +600,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 10입(7+3) - 스페셜 기프트 에디션 (공식수입)</t>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 7입 - 단독 기프트박스 증정 (공식수입)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -610,14 +610,14 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>43,000원</t>
+          <t>34,000원</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -631,7 +631,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[그레인온] 골드 카무트 브랜드밀효소G 3개월분+10포증정(총100포)+프리미엄90 5포 추가증정</t>
+          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)+파인키위효소 1개월+저당견과류바</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -641,14 +641,14 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>20,000원</t>
+          <t>43,700원</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>1.6</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -657,26 +657,26 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>"선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 1입 추가 증정</t>
+          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>아일로</t>
+          <t>그레인온</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>65,900원</t>
+          <t>42,900원</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
@@ -688,29 +688,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>멀티비타민/종합비타민</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 30입 - 시그니처 기프트 에디션 (공식수입)</t>
+          <t>[그레인온] 골드 카무트 브랜드밀효소G 3개월분+10포증정(총100포)+프리미엄90 5포 추가증정</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>오쏘몰</t>
+          <t>그레인온</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>109,000원</t>
+          <t>20,980원</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -719,26 +719,26 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 7입 (공식수입)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>단독</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>34,900원</t>
+          <t>34,000원</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
@@ -755,24 +755,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[센트룸] 맛있는 멀티비타민 미네랄 멀티구미 (80구미)</t>
+          <t>옵티젠 이뮨 멀티비타민&amp;미네랄 10입 / 1박스 (+GIFT 쇼핑백)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>센트룸</t>
+          <t>옵티젠</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>24,000원</t>
+          <t>26,900원</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>5</v>
+        <v>2.17</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -790,8 +790,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
@@ -846,17 +846,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
+          <t>바나바잎 10정 10일분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>1,000원</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -877,17 +877,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>동국 맛있는 센시안 브이캔디 20정 20일분</t>
+          <t>신상 NEW</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>다이소</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -903,17 +903,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>멀티비타민/종합비타민</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>브이팩 남성용 올인원 멀티 비타민 7포</t>
+          <t>유기농 엑스트라버진 올리브오일 10포</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>안국약품</t>
+          <t>홀베리</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -922,7 +922,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -934,29 +934,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>데일리와이즈 혈당컷 다이어트 12정 12일분</t>
+          <t>동국 맛있는 센시안 브이캔디 20정 20일분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>종근당</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -965,29 +965,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>비타민D</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>비타민D 4000IU 30정 30일분</t>
+          <t>데일리와이즈 혈당컷 다이어트 12정 12일분</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>종근당</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -996,26 +996,26 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>rTG 오메가3 30캡슐 30일분</t>
+          <t>건강식품</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>다이소</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
@@ -1027,17 +1027,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>운동부스터 생유산균 스틱 5포 5일분</t>
+          <t>정성담은 배도라지스틱 12포</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>유한양행</t>
+          <t>자연관</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1046,7 +1046,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
@@ -1058,29 +1058,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>마그네슘</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>마그네슘 30정 30일분</t>
+          <t>데일리와이즈 푸룬 구미 7일분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>종근당</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>1,000원</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>3.5</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>콜린 미오이노시톨 4000 10포</t>
+          <t>이지슬로 엑스트라버진 올리브오일＆레몬 4병</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>안국약품</t>
+          <t>자연관</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1108,7 +1108,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
@@ -1125,24 +1125,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>동국 맛있는 샐러드 미니볼 15포 15일분</t>
+          <t>콜린 미오이노시톨 4000 10포</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>안국약품</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1161,9 +1161,9 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
   </cols>
@@ -1211,29 +1211,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[올영단독] 닥터린 파비플로라 알파CD 프리미엄 10g X 30포 (1개월분)</t>
+          <t>[웰니스 루틴] 온리추얼 슬리밍컷 다이어트/리셋 브이라인/글로우업 콜라겐 7포(+1포)/14포 (8/14일분)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>닥터린</t>
+          <t>온리추얼</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>19,070원</t>
+          <t>11,900원</t>
         </is>
       </c>
       <c r="F2" t="n">
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -1242,29 +1242,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>비타민C/항산화</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균) + 철분 헤모케어 3포 증정</t>
+          <t>고려은단 비타민C1000 이지+비타민D 120정 (60일분)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>덴프스</t>
+          <t>고려은단</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>37,050원</t>
+          <t>10,900원</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -1273,26 +1273,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>비타민C/항산화</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[올영단독] 지노마스터 질유산균 70캡슐 (70일분)</t>
+          <t>고려은단 비타민C1000 600정 (20개월분)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>지노마스터</t>
+          <t>고려은단</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>59,000원</t>
+          <t>42,900원</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
@@ -1309,21 +1309,21 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[6월 올영픽/곽민경 PICK] 생활약속 기분전환 알파플러스 10포 (+1포 증정기획)</t>
+          <t>CJ 한뿌리 흑삼지천보 진녹 30포 (1개월분) (온)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>생활약속</t>
+          <t>한뿌리</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>15,400원</t>
+          <t>250,000원</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -1354,10 +1354,10 @@
         </is>
       </c>
       <c r="F6" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G6" t="n">
         <v>5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -1366,29 +1366,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>프로뉴트리션 듀얼플랜 다이어트 유산균 14포</t>
+          <t>레놉티 시너업글로우 14포 (14일분)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>프로뉴트리션</t>
+          <t>레놉티</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>35,800원</t>
+          <t>32,200원</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -1397,26 +1397,26 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>프로바이오틱스/유산균</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>한삼인 잠잠 6개입 (6일분)</t>
+          <t>[호빵맨콜라보] 이너플로라 질유산균 60캡슐+호빵맨 스티커 / 이노시톨콜린 30포</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>한삼인</t>
+          <t>뉴오리진</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>27,000원</t>
+          <t>38,900원</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
@@ -1428,26 +1428,26 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>[6월 올영픽/골라담기] CJ웰케어 건강루틴 가격혁명 10종 택 1</t>
+          <t>[서현PICK] 콜레올로지 PRO 600mg*30/60정 단품</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>씨제이웰케어</t>
+          <t>푸드올로지</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5,900원</t>
+          <t>17,400원</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
@@ -1459,29 +1459,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[포켓몬 에디션] 덴마크 유산균이야기 30캡슐 1+1 (+꼬부기 러기지택) (60일분)</t>
+          <t>고려은단 메가도스 이뮨샷 4개입 (4일분)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>덴프스</t>
+          <t>고려은단</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>30,400원</t>
+          <t>9,900원</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -1490,29 +1490,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>프로바이오틱스/유산균</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>탄탄 더블컷 다이어트 젤리 3종 택1 (믹스베리맛/자두맛/애플유자맛)</t>
+          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균) + 철분 헤모케어 3포 증정</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>탄탄</t>
+          <t>덴프스</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>9,900원</t>
+          <t>37,050원</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>10</v>
+        <v>5.2</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1576,16 +1576,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>13.3</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -1598,10 +1598,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>6.7</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -1610,7 +1610,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1620,16 +1620,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -1642,16 +1642,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -1664,16 +1664,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -1730,13 +1730,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>20</v>
+        <v>13.3</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
         <v>2</v>
@@ -1752,19 +1752,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C10" t="n">
-        <v>13.3</v>
+        <v>6.7</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -1774,13 +1774,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" t="n">
-        <v>6.7</v>
+        <v>3.3</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
@@ -1796,19 +1796,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C12" t="n">
-        <v>30</v>
+        <v>56.7</v>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F12" t="n">
         <v>3</v>
-      </c>
-      <c r="F12" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
data: 2026-07 월별 취합
</commit_message>
<xml_diff>
--- a/data/monthly/2026-06_월별취합.xlsx
+++ b/data/monthly/2026-06_월별취합.xlsx
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,37 +441,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>순위(월평균)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>평균가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>평균순위</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>등장횟수</t>
         </is>
@@ -799,37 +811,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>순위(월평균)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>평균가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>평균순위</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>등장횟수</t>
         </is>
@@ -1169,37 +1181,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>순위(월평균)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>평균가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>평균순위</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>등장횟수</t>
         </is>
@@ -1538,32 +1550,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>

</xml_diff>

<commit_message>
refactor: data/daily 월별 하위폴더 구조 도입
- main.py, app.py: 저장 경로에 today[:7] 월 폴더 자동 추가
- monthly_aggregate.py: 집계 대상 월 폴더에서만 파일 탐색
- 기존 daily xlsx 7개 월별 폴더로 이동
- 설계서.md, README.md 파일 구조 표기 갱신
</commit_message>
<xml_diff>
--- a/data/monthly/2026-06_월별취합.xlsx
+++ b/data/monthly/2026-06_월별취합.xlsx
@@ -20,16 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -441,37 +429,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>순위(월평균)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>평균가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>평균순위</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>등장횟수</t>
         </is>
@@ -811,37 +799,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>순위(월평균)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>평균가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>평균순위</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>등장횟수</t>
         </is>
@@ -1181,37 +1169,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>순위(월평균)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>평균가격</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>평균순위</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>등장횟수</t>
         </is>
@@ -1550,32 +1538,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>

</xml_diff>